<commit_message>
update logs with missing data
</commit_message>
<xml_diff>
--- a/qc/spreadsheets/socialdoors_qc.xlsx
+++ b/qc/spreadsheets/socialdoors_qc.xlsx
@@ -466,8 +466,8 @@
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="45" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="45" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
     <col width="45" customWidth="1" min="22" max="22"/>
     <col width="45" customWidth="1" min="23" max="23"/>
     <col width="45" customWidth="1" min="24" max="24"/>
@@ -30483,6 +30483,12 @@
           <t>1</t>
         </is>
       </c>
+      <c r="F328" t="n">
+        <v>42.03156019002199</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0.1921243113308369</v>
+      </c>
       <c r="H328" t="n">
         <v>54</v>
       </c>
@@ -30498,6 +30504,12 @@
       <c r="L328" t="n">
         <v>99.58286837770339</v>
       </c>
+      <c r="M328" t="b">
+        <v>0</v>
+      </c>
+      <c r="N328" t="b">
+        <v>0</v>
+      </c>
       <c r="O328" t="b">
         <v>0</v>
       </c>
@@ -30508,21 +30520,21 @@
         <v>0</v>
       </c>
       <c r="S328" t="b">
-        <v>0</v>
-      </c>
-      <c r="T328" t="inlineStr">
-        <is>
-          <t>fd_mean:missing_mriqc_json;tsnr:missing_mriqc_json</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="U328" t="inlineStr">
         <is>
-          <t>incomplete</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V328" t="inlineStr">
         <is>
           <t>bids/sub-11078/ses-02/func/sub-11078_ses-02_task-doors_run-1_echo-2_part-mag_bold.nii.gz</t>
+        </is>
+      </c>
+      <c r="W328" t="inlineStr">
+        <is>
+          <t>derivatives/mriqc/sub-11078/ses-02/func/sub-11078_ses-02_task-doors_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X328" t="inlineStr">
@@ -30562,6 +30574,12 @@
           <t>1</t>
         </is>
       </c>
+      <c r="F329" t="n">
+        <v>52.43493898306042</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0.1863534513295579</v>
+      </c>
       <c r="H329" t="n">
         <v>41</v>
       </c>
@@ -30577,6 +30595,12 @@
       <c r="L329" t="n">
         <v>99.62670705138424</v>
       </c>
+      <c r="M329" t="b">
+        <v>0</v>
+      </c>
+      <c r="N329" t="b">
+        <v>0</v>
+      </c>
       <c r="O329" t="b">
         <v>0</v>
       </c>
@@ -30587,21 +30611,21 @@
         <v>0</v>
       </c>
       <c r="S329" t="b">
-        <v>0</v>
-      </c>
-      <c r="T329" t="inlineStr">
-        <is>
-          <t>fd_mean:missing_mriqc_json;tsnr:missing_mriqc_json</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="U329" t="inlineStr">
         <is>
-          <t>incomplete</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V329" t="inlineStr">
         <is>
           <t>bids/sub-11078/ses-02/func/sub-11078_ses-02_task-socialdoors_run-1_echo-2_part-mag_bold.nii.gz</t>
+        </is>
+      </c>
+      <c r="W329" t="inlineStr">
+        <is>
+          <t>derivatives/mriqc/sub-11078/ses-02/func/sub-11078_ses-02_task-socialdoors_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X329" t="inlineStr">
@@ -67125,7 +67149,7 @@
     <col width="31" customWidth="1" min="9" max="9"/>
     <col width="27" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
@@ -76783,15 +76807,22 @@
         <v>0</v>
       </c>
       <c r="J166" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K166" t="b">
-        <v>0</v>
-      </c>
-      <c r="L166" t="inlineStr">
-        <is>
-          <t>socialdoors_qc_incomplete;doors_qc_incomplete</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="M166" t="n">
+        <v>52.43493898306042</v>
+      </c>
+      <c r="N166" t="n">
+        <v>42.03156019002199</v>
+      </c>
+      <c r="O166" t="n">
+        <v>0.1863534513295579</v>
+      </c>
+      <c r="P166" t="n">
+        <v>0.1921243113308369</v>
       </c>
       <c r="Q166" t="n">
         <v>20</v>
@@ -88671,22 +88702,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="E2" t="n">
-        <v>27.1302936442662</v>
+        <v>27.13098336174153</v>
       </c>
       <c r="F2" t="n">
-        <v>40.56536435434828</v>
+        <v>40.61143377644476</v>
       </c>
       <c r="G2" t="n">
-        <v>13.43507071008207</v>
+        <v>13.48045041470323</v>
       </c>
       <c r="H2" t="n">
-        <v>6.977687579143094</v>
+        <v>6.910307739686687</v>
       </c>
       <c r="I2" t="n">
-        <v>60.71797041947138</v>
+        <v>60.8321093984996</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -88714,22 +88745,22 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1192655314693145</v>
+        <v>0.1193515892481275</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2253169963265305</v>
+        <v>0.2252637507353653</v>
       </c>
       <c r="G3" t="n">
-        <v>0.106051464857216</v>
+        <v>0.1059121614872377</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.03981166581650948</v>
+        <v>-0.03951665298272904</v>
       </c>
       <c r="I3" t="n">
-        <v>0.3843941936123545</v>
+        <v>0.3841319929662218</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>

</xml_diff>